<commit_message>
Refactor build_activity_tracker.py to streamline activity tracker generation
Remove the legend and usage instructions from the `build_activity_tracker.py` script to simplify the output. This change focuses on enhancing the clarity and efficiency of the activity tracker generation process, while maintaining the core functionality of consolidating priority actions and deadlines.
</commit_message>
<xml_diff>
--- a/opportunities/activity_tracker.xlsx
+++ b/opportunities/activity_tracker.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,11 +35,6 @@
     </font>
     <font>
       <name val="Calibri"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -102,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -118,10 +113,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -488,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1287,33 +1278,8 @@
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>How to use</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="40" customHeight="1">
-      <c r="A22" s="7" t="inlineStr">
-        <is>
-          <t>Priority 1 = do today. Priority 2 = this week / before deadline. Priority 3 = later. Done = already applied or finished. Update the Status column as you finish (To do -&gt; Doing -&gt; Done).</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Built 2026-08-11 10:24 from tracker.xlsx + new_grants.xlsx. Rebuild: python opportunities/build_activity_tracker.py</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:H19"/>
-  <mergeCells count="2">
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="A22:H22"/>
-  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>